<commit_message>
feat(pricing): add retailer-controlled inventory discounts
</commit_message>
<xml_diff>
--- a/data/inventory.xlsx
+++ b/data/inventory.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R31"/>
+  <dimension ref="A1:U31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,55 +454,70 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>discount_mode</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>discount_pct</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>show_discount</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>stock_qty</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>surplus_reason</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>days_in_surplus</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>expiry_date</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>sizes</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>colours</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>tags</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>dietary</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>allergens</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>condition</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>active</t>
         </is>
@@ -538,43 +553,54 @@
         <v>89.90000000000001</v>
       </c>
       <c r="G2" t="n">
-        <v>61.13</v>
-      </c>
-      <c r="H2" t="n">
+        <v>89.90000000000001</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>protected</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="b">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
         <v>7</v>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>season_end</t>
         </is>
       </c>
-      <c r="J2" t="n">
+      <c r="M2" t="n">
         <v>17</v>
       </c>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr">
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr">
         <is>
           <t>S|M|L</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>black|olive</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>bold|edgy|fashion|practical|adventurous|streetwear</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="R2" t="b">
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="U2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -608,43 +634,54 @@
         <v>58</v>
       </c>
       <c r="G3" t="n">
-        <v>39.44</v>
-      </c>
-      <c r="H3" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>markdown</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>20</v>
+      </c>
+      <c r="J3" t="b">
+        <v>1</v>
+      </c>
+      <c r="K3" t="n">
         <v>9</v>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>overproduction</t>
         </is>
       </c>
-      <c r="J3" t="n">
+      <c r="M3" t="n">
         <v>24</v>
       </c>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr">
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr">
         <is>
           <t>S|M|L</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>oat|forest_green</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>cozy|classic|fashion|comfort|natural|clean</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="R3" t="b">
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="U3" t="b">
         <v>1</v>
       </c>
     </row>
@@ -678,43 +715,54 @@
         <v>32</v>
       </c>
       <c r="G4" t="n">
-        <v>21.76</v>
-      </c>
-      <c r="H4" t="n">
+        <v>24</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>markdown</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>25</v>
+      </c>
+      <c r="J4" t="b">
+        <v>1</v>
+      </c>
+      <c r="K4" t="n">
         <v>14</v>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>surplus_stock</t>
         </is>
       </c>
-      <c r="J4" t="n">
+      <c r="M4" t="n">
         <v>31</v>
       </c>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr">
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr">
         <is>
           <t>ONE_SIZE</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>natural|colourful</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>practical|minimal|fashion|portable|shareable|playful</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="R4" t="b">
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="U4" t="b">
         <v>1</v>
       </c>
     </row>
@@ -748,43 +796,54 @@
         <v>69.90000000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>47.53</v>
-      </c>
-      <c r="H5" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>protected</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="b">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
         <v>4</v>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>season_end</t>
         </is>
       </c>
-      <c r="J5" t="n">
+      <c r="M5" t="n">
         <v>38</v>
       </c>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr">
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr">
         <is>
           <t>S|M</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>charcoal|beige</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>classic|clean|fashion|practical|minimal</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="R5" t="b">
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="U5" t="b">
         <v>1</v>
       </c>
     </row>
@@ -818,43 +877,54 @@
         <v>49.9</v>
       </c>
       <c r="G6" t="n">
-        <v>33.93</v>
-      </c>
-      <c r="H6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I6" t="inlineStr">
+        <v>49.9</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>protected</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="b">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>1</v>
+      </c>
+      <c r="L6" t="inlineStr">
         <is>
           <t>deadstock</t>
         </is>
       </c>
-      <c r="J6" t="n">
+      <c r="M6" t="n">
         <v>45</v>
       </c>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr">
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr">
         <is>
           <t>XXS</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>neon_yellow</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>edgy|dark|fashion|bold|niche|rave</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="R6" t="b">
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="U6" t="b">
         <v>0</v>
       </c>
     </row>
@@ -888,39 +958,50 @@
         <v>28</v>
       </c>
       <c r="G7" t="n">
-        <v>19.04</v>
-      </c>
-      <c r="H7" t="n">
+        <v>22.4</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>markdown</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>20</v>
+      </c>
+      <c r="J7" t="b">
+        <v>1</v>
+      </c>
+      <c r="K7" t="n">
         <v>12</v>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>repackaging</t>
         </is>
       </c>
-      <c r="J7" t="n">
+      <c r="M7" t="n">
         <v>52</v>
       </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr">
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr">
         <is>
           <t>berry|rose</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="Q7" t="inlineStr">
         <is>
           <t>bold|colourful|beauty|portable|playful|cute</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="R7" t="b">
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="U7" t="b">
         <v>1</v>
       </c>
     </row>
@@ -954,39 +1035,50 @@
         <v>42</v>
       </c>
       <c r="G8" t="n">
-        <v>28.56</v>
-      </c>
-      <c r="H8" t="n">
+        <v>42</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>protected</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="b">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
         <v>8</v>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>overstock</t>
         </is>
       </c>
-      <c r="J8" t="n">
+      <c r="M8" t="n">
         <v>59</v>
       </c>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr">
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr">
         <is>
           <t>clear</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="Q8" t="inlineStr">
         <is>
           <t>clean|calm|beauty|natural|practical|skincare</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="R8" t="b">
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="U8" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1020,39 +1112,50 @@
         <v>34</v>
       </c>
       <c r="G9" t="n">
-        <v>23.12</v>
-      </c>
-      <c r="H9" t="n">
+        <v>34</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>protected</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
         <v>10</v>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>season_end</t>
         </is>
       </c>
-      <c r="J9" t="n">
+      <c r="M9" t="n">
         <v>66</v>
       </c>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr">
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr">
         <is>
           <t>green</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="Q9" t="inlineStr">
         <is>
           <t>calm|natural|beauty|cozy|clean|skincare</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="R9" t="b">
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr"/>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="U9" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1086,39 +1189,50 @@
         <v>22</v>
       </c>
       <c r="G10" t="n">
-        <v>14.96</v>
-      </c>
-      <c r="H10" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>markdown</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>15</v>
+      </c>
+      <c r="J10" t="b">
+        <v>1</v>
+      </c>
+      <c r="K10" t="n">
         <v>16</v>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>packaging_update</t>
         </is>
       </c>
-      <c r="J10" t="n">
+      <c r="M10" t="n">
         <v>73</v>
       </c>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr">
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr">
         <is>
           <t>yellow|white</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="Q10" t="inlineStr">
         <is>
           <t>cute|portable|beauty|natural|clean|shareable</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="R10" t="b">
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="U10" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1152,47 +1266,58 @@
         <v>15</v>
       </c>
       <c r="G11" t="n">
-        <v>8.25</v>
-      </c>
-      <c r="H11" t="n">
+        <v>9.75</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>markdown</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>35</v>
+      </c>
+      <c r="J11" t="b">
+        <v>1</v>
+      </c>
+      <c r="K11" t="n">
         <v>18</v>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>short_shelf_life</t>
         </is>
       </c>
-      <c r="J11" t="n">
+      <c r="M11" t="n">
         <v>80</v>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr">
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr">
         <is>
           <t>food|shareable|adventurous|bold|vegan</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr">
+      <c r="R11" t="inlineStr">
         <is>
           <t>vegan|gluten_free</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr">
+      <c r="S11" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="R11" t="b">
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="U11" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1226,47 +1351,58 @@
         <v>22</v>
       </c>
       <c r="G12" t="n">
-        <v>12.1</v>
-      </c>
-      <c r="H12" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>markdown</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>25</v>
+      </c>
+      <c r="J12" t="b">
+        <v>1</v>
+      </c>
+      <c r="K12" t="n">
         <v>13</v>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>overproduction</t>
         </is>
       </c>
-      <c r="J12" t="n">
+      <c r="M12" t="n">
         <v>11</v>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr">
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr">
         <is>
           <t>food|energetic|adventurous|portable|vegan</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr">
+      <c r="R12" t="inlineStr">
         <is>
           <t>vegan|halal</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr">
+      <c r="S12" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="R12" t="b">
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="U12" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1300,47 +1436,58 @@
         <v>18</v>
       </c>
       <c r="G13" t="n">
-        <v>9.9</v>
-      </c>
-      <c r="H13" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>markdown</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>30</v>
+      </c>
+      <c r="J13" t="b">
+        <v>1</v>
+      </c>
+      <c r="K13" t="n">
         <v>5</v>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>daily_surplus</t>
         </is>
       </c>
-      <c r="J13" t="n">
+      <c r="M13" t="n">
         <v>18</v>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr">
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr">
         <is>
           <t>food|cozy|comfort|shareable|classic</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr">
+      <c r="R13" t="inlineStr">
         <is>
           <t>vegetarian</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr">
+      <c r="S13" t="inlineStr">
         <is>
           <t>gluten|milk|nuts</t>
         </is>
       </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="R13" t="b">
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="U13" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1374,47 +1521,58 @@
         <v>19</v>
       </c>
       <c r="G14" t="n">
-        <v>10.45</v>
-      </c>
-      <c r="H14" t="n">
+        <v>14.25</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>markdown</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>25</v>
+      </c>
+      <c r="J14" t="b">
+        <v>1</v>
+      </c>
+      <c r="K14" t="n">
         <v>11</v>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>short_shelf_life</t>
         </is>
       </c>
-      <c r="J14" t="n">
+      <c r="M14" t="n">
         <v>25</v>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr">
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr">
         <is>
           <t>food|practical|shareable|playful|vegan</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr">
+      <c r="R14" t="inlineStr">
         <is>
           <t>vegan</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr">
+      <c r="S14" t="inlineStr">
         <is>
           <t>gluten</t>
         </is>
       </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="R14" t="b">
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="U14" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1448,47 +1606,58 @@
         <v>21</v>
       </c>
       <c r="G15" t="n">
-        <v>11.55</v>
-      </c>
-      <c r="H15" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>markdown</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>20</v>
+      </c>
+      <c r="J15" t="b">
+        <v>1</v>
+      </c>
+      <c r="K15" t="n">
         <v>9</v>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>surplus_stock</t>
         </is>
       </c>
-      <c r="J15" t="n">
+      <c r="M15" t="n">
         <v>32</v>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr">
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr">
         <is>
           <t>food|practical|natural|shareable|vegan</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr">
+      <c r="R15" t="inlineStr">
         <is>
           <t>vegan</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr">
+      <c r="S15" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="R15" t="b">
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="U15" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1522,39 +1691,50 @@
         <v>32</v>
       </c>
       <c r="G16" t="n">
-        <v>21.76</v>
-      </c>
-      <c r="H16" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>markdown</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>20</v>
+      </c>
+      <c r="J16" t="b">
+        <v>1</v>
+      </c>
+      <c r="K16" t="n">
         <v>6</v>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="L16" t="inlineStr">
         <is>
           <t>season_end</t>
         </is>
       </c>
-      <c r="J16" t="n">
+      <c r="M16" t="n">
         <v>39</v>
       </c>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr">
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr">
         <is>
           <t>green|terracotta</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr">
+      <c r="Q16" t="inlineStr">
         <is>
           <t>natural|calm|home|decorative|playful|slow</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr"/>
-      <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="R16" t="b">
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="U16" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1588,39 +1768,50 @@
         <v>48</v>
       </c>
       <c r="G17" t="n">
-        <v>32.64</v>
-      </c>
-      <c r="H17" t="n">
+        <v>48</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>protected</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="b">
+        <v>0</v>
+      </c>
+      <c r="K17" t="n">
         <v>5</v>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="L17" t="inlineStr">
         <is>
           <t>overproduction</t>
         </is>
       </c>
-      <c r="J17" t="n">
+      <c r="M17" t="n">
         <v>46</v>
       </c>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr">
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr">
         <is>
           <t>navy|sand</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr">
+      <c r="Q17" t="inlineStr">
         <is>
           <t>cozy|portable|comfort|practical|calm|adventurous</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="R17" t="b">
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="U17" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1654,39 +1845,50 @@
         <v>26</v>
       </c>
       <c r="G18" t="n">
-        <v>17.68</v>
-      </c>
-      <c r="H18" t="n">
+        <v>22.1</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>markdown</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>15</v>
+      </c>
+      <c r="J18" t="b">
+        <v>0</v>
+      </c>
+      <c r="K18" t="n">
         <v>8</v>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>packaging_update</t>
         </is>
       </c>
-      <c r="J18" t="n">
+      <c r="M18" t="n">
         <v>53</v>
       </c>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr">
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr">
         <is>
           <t>lavender</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr">
+      <c r="Q18" t="inlineStr">
         <is>
           <t>calm|cozy|natural|beauty|shareable|slow</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="R18" t="b">
+      <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="U18" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1720,39 +1922,50 @@
         <v>36</v>
       </c>
       <c r="G19" t="n">
-        <v>24.48</v>
-      </c>
-      <c r="H19" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>markdown</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>20</v>
+      </c>
+      <c r="J19" t="b">
+        <v>1</v>
+      </c>
+      <c r="K19" t="n">
         <v>10</v>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>discontinued_colour</t>
         </is>
       </c>
-      <c r="J19" t="n">
+      <c r="M19" t="n">
         <v>60</v>
       </c>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr">
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr">
         <is>
           <t>blue|silver</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr">
+      <c r="Q19" t="inlineStr">
         <is>
           <t>practical|portable|energetic|natural|shareable</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="R19" t="b">
+      <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr"/>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="U19" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1786,39 +1999,50 @@
         <v>32</v>
       </c>
       <c r="G20" t="n">
-        <v>21.76</v>
-      </c>
-      <c r="H20" t="n">
+        <v>32</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>protected</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" t="b">
+        <v>0</v>
+      </c>
+      <c r="K20" t="n">
         <v>9</v>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>packaging_update</t>
         </is>
       </c>
-      <c r="J20" t="n">
+      <c r="M20" t="n">
         <v>67</v>
       </c>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr">
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr">
         <is>
           <t>amber|cream</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr">
+      <c r="Q20" t="inlineStr">
         <is>
           <t>cozy|calm|home|decorative|natural|slow</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="R20" t="b">
+      <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="U20" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1852,39 +2076,50 @@
         <v>38</v>
       </c>
       <c r="G21" t="n">
-        <v>25.84</v>
-      </c>
-      <c r="H21" t="n">
+        <v>38</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>protected</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" t="b">
+        <v>0</v>
+      </c>
+      <c r="K21" t="n">
         <v>5</v>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>minor_packaging_damage</t>
         </is>
       </c>
-      <c r="J21" t="n">
+      <c r="M21" t="n">
         <v>74</v>
       </c>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr">
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr">
         <is>
           <t>terracotta|sand</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr">
+      <c r="Q21" t="inlineStr">
         <is>
           <t>minimal|cozy|home|practical|classic</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="R21" t="b">
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="U21" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1918,39 +2153,50 @@
         <v>44</v>
       </c>
       <c r="G22" t="n">
-        <v>29.92</v>
-      </c>
-      <c r="H22" t="n">
+        <v>44</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>protected</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" t="b">
+        <v>0</v>
+      </c>
+      <c r="K22" t="n">
         <v>3</v>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="L22" t="inlineStr">
         <is>
           <t>display_refresh</t>
         </is>
       </c>
-      <c r="J22" t="n">
+      <c r="M22" t="n">
         <v>81</v>
       </c>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr">
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr">
         <is>
           <t>speckled|cream</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr">
+      <c r="Q22" t="inlineStr">
         <is>
           <t>bold|decorative|home|practical|minimal</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr"/>
-      <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="R22" t="b">
+      <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="U22" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1984,39 +2230,50 @@
         <v>28</v>
       </c>
       <c r="G23" t="n">
-        <v>19.04</v>
-      </c>
-      <c r="H23" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>markdown</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>15</v>
+      </c>
+      <c r="J23" t="b">
+        <v>1</v>
+      </c>
+      <c r="K23" t="n">
         <v>12</v>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="L23" t="inlineStr">
         <is>
           <t>surplus_stock</t>
         </is>
       </c>
-      <c r="J23" t="n">
+      <c r="M23" t="n">
         <v>12</v>
       </c>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr">
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr">
         <is>
           <t>clear|smoke</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr">
+      <c r="Q23" t="inlineStr">
         <is>
           <t>minimal|portable|home|shareable|practical</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr"/>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="R23" t="b">
+      <c r="R23" t="inlineStr"/>
+      <c r="S23" t="inlineStr"/>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="U23" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2050,39 +2307,50 @@
         <v>59.9</v>
       </c>
       <c r="G24" t="n">
-        <v>40.73</v>
-      </c>
-      <c r="H24" t="n">
+        <v>44.92</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>markdown</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>25</v>
+      </c>
+      <c r="J24" t="b">
+        <v>1</v>
+      </c>
+      <c r="K24" t="n">
         <v>6</v>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="L24" t="inlineStr">
         <is>
           <t>discontinued_colour</t>
         </is>
       </c>
-      <c r="J24" t="n">
+      <c r="M24" t="n">
         <v>19</v>
       </c>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr">
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr">
         <is>
           <t>matte_black|white</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr">
+      <c r="Q24" t="inlineStr">
         <is>
           <t>tech|portable|energetic|dark|audio</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="R24" t="b">
+      <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="U24" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2116,39 +2384,50 @@
         <v>45</v>
       </c>
       <c r="G25" t="n">
-        <v>30.6</v>
-      </c>
-      <c r="H25" t="n">
+        <v>36</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>markdown</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>20</v>
+      </c>
+      <c r="J25" t="b">
+        <v>1</v>
+      </c>
+      <c r="K25" t="n">
         <v>7</v>
       </c>
-      <c r="I25" t="inlineStr">
+      <c r="L25" t="inlineStr">
         <is>
           <t>overstock</t>
         </is>
       </c>
-      <c r="J25" t="n">
+      <c r="M25" t="n">
         <v>26</v>
       </c>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr">
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr">
         <is>
           <t>sage_green|black</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr">
+      <c r="Q25" t="inlineStr">
         <is>
           <t>tech|portable|practical|adventurous</t>
         </is>
       </c>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="R25" t="b">
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr"/>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="U25" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2182,39 +2461,50 @@
         <v>19</v>
       </c>
       <c r="G26" t="n">
-        <v>12.92</v>
-      </c>
-      <c r="H26" t="n">
+        <v>16.15</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>markdown</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
         <v>15</v>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="J26" t="b">
+        <v>1</v>
+      </c>
+      <c r="K26" t="n">
+        <v>15</v>
+      </c>
+      <c r="L26" t="inlineStr">
         <is>
           <t>overproduction</t>
         </is>
       </c>
-      <c r="J26" t="n">
+      <c r="M26" t="n">
         <v>33</v>
       </c>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr">
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr">
         <is>
           <t>black|colourful</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr">
+      <c r="Q26" t="inlineStr">
         <is>
           <t>tech|practical|portable|clean|shareable</t>
         </is>
       </c>
-      <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr"/>
-      <c r="Q26" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="R26" t="b">
+      <c r="R26" t="inlineStr"/>
+      <c r="S26" t="inlineStr"/>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="U26" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2248,39 +2538,50 @@
         <v>89</v>
       </c>
       <c r="G27" t="n">
-        <v>60.52</v>
-      </c>
-      <c r="H27" t="n">
-        <v>1</v>
-      </c>
-      <c r="I27" t="inlineStr">
+        <v>89</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>protected</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" t="b">
+        <v>0</v>
+      </c>
+      <c r="K27" t="n">
+        <v>1</v>
+      </c>
+      <c r="L27" t="inlineStr">
         <is>
           <t>discontinued_model</t>
         </is>
       </c>
-      <c r="J27" t="n">
+      <c r="M27" t="n">
         <v>40</v>
       </c>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr">
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr">
         <is>
           <t>black</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr">
+      <c r="Q27" t="inlineStr">
         <is>
           <t>tech|audio|dark|edgy|niche</t>
         </is>
       </c>
-      <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr"/>
-      <c r="Q27" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="R27" t="b">
+      <c r="R27" t="inlineStr"/>
+      <c r="S27" t="inlineStr"/>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="U27" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2314,39 +2615,50 @@
         <v>26</v>
       </c>
       <c r="G28" t="n">
-        <v>17.68</v>
-      </c>
-      <c r="H28" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>markdown</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>20</v>
+      </c>
+      <c r="J28" t="b">
+        <v>1</v>
+      </c>
+      <c r="K28" t="n">
         <v>13</v>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="L28" t="inlineStr">
         <is>
           <t>season_end</t>
         </is>
       </c>
-      <c r="J28" t="n">
+      <c r="M28" t="n">
         <v>47</v>
       </c>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr">
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr">
         <is>
           <t>forest_green|cream</t>
         </is>
       </c>
-      <c r="N28" t="inlineStr">
+      <c r="Q28" t="inlineStr">
         <is>
           <t>stationery|calm|practical|minimal|clean</t>
         </is>
       </c>
-      <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr"/>
-      <c r="Q28" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="R28" t="b">
+      <c r="R28" t="inlineStr"/>
+      <c r="S28" t="inlineStr"/>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="U28" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2380,39 +2692,50 @@
         <v>16</v>
       </c>
       <c r="G29" t="n">
-        <v>10.88</v>
-      </c>
-      <c r="H29" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>markdown</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>10</v>
+      </c>
+      <c r="J29" t="b">
+        <v>1</v>
+      </c>
+      <c r="K29" t="n">
         <v>20</v>
       </c>
-      <c r="I29" t="inlineStr">
+      <c r="L29" t="inlineStr">
         <is>
           <t>surplus_stock</t>
         </is>
       </c>
-      <c r="J29" t="n">
+      <c r="M29" t="n">
         <v>54</v>
       </c>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr">
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr">
         <is>
           <t>colourful|natural</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr">
+      <c r="Q29" t="inlineStr">
         <is>
           <t>stationery|playful|practical|colourful|shareable</t>
         </is>
       </c>
-      <c r="O29" t="inlineStr"/>
-      <c r="P29" t="inlineStr"/>
-      <c r="Q29" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="R29" t="b">
+      <c r="R29" t="inlineStr"/>
+      <c r="S29" t="inlineStr"/>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="U29" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2446,39 +2769,50 @@
         <v>52</v>
       </c>
       <c r="G30" t="n">
-        <v>35.36</v>
-      </c>
-      <c r="H30" t="n">
+        <v>52</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>protected</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" t="b">
+        <v>0</v>
+      </c>
+      <c r="K30" t="n">
         <v>4</v>
       </c>
-      <c r="I30" t="inlineStr">
+      <c r="L30" t="inlineStr">
         <is>
           <t>display_refresh</t>
         </is>
       </c>
-      <c r="J30" t="n">
+      <c r="M30" t="n">
         <v>61</v>
       </c>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr">
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr">
         <is>
           <t>blue|coral|cream</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr">
+      <c r="Q30" t="inlineStr">
         <is>
           <t>stationery|bold|colourful|practical|decorative</t>
         </is>
       </c>
-      <c r="O30" t="inlineStr"/>
-      <c r="P30" t="inlineStr"/>
-      <c r="Q30" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="R30" t="b">
+      <c r="R30" t="inlineStr"/>
+      <c r="S30" t="inlineStr"/>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="U30" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2512,39 +2846,50 @@
         <v>24</v>
       </c>
       <c r="G31" t="n">
-        <v>16.32</v>
-      </c>
-      <c r="H31" t="n">
+        <v>24</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>protected</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" t="b">
+        <v>0</v>
+      </c>
+      <c r="K31" t="n">
         <v>7</v>
       </c>
-      <c r="I31" t="inlineStr">
+      <c r="L31" t="inlineStr">
         <is>
           <t>packaging_update</t>
         </is>
       </c>
-      <c r="J31" t="n">
+      <c r="M31" t="n">
         <v>68</v>
       </c>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr">
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr">
         <is>
           <t>brass|black</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr">
+      <c r="Q31" t="inlineStr">
         <is>
           <t>stationery|minimal|classic|decorative|shareable</t>
         </is>
       </c>
-      <c r="O31" t="inlineStr"/>
-      <c r="P31" t="inlineStr"/>
-      <c r="Q31" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="R31" t="b">
+      <c r="R31" t="inlineStr"/>
+      <c r="S31" t="inlineStr"/>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="U31" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>